<commit_message>
Update Nunes to published version (Res Sports Med, pp.170-184) + corrected matrix
</commit_message>
<xml_diff>
--- a/LR_Matrix_v2.xlsx
+++ b/LR_Matrix_v2.xlsx
@@ -641,9 +641,9 @@
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>• ★ "The results highlighted that the same SSCG practice context, applied to different age groups, promoted different response outcomes from participants. Greater changes were demonstrated in younger age groups and on larger pitches." (p. 170)
-• "young children should not be treated as 'mini-adults' and have different needs and capacities, compared to older age group athletes." (p. 175)
-• "The use of smaller playing areas seems to favour the increase of passing actions in older players while … increases in playing area appear to alter the available time for younger players to practice skills without the major constraint of pressing." (p. 176)</t>
+          <t>• [⑰] ★ "Results showed higher values in the large playing area for under-11 in the distance covered in different speed zones, sprint number and RPE (all p &lt; .001) … Opposite, under-23s were able to perform more passing on smaller playing areas … The impact of different playing areas was reduced for the under-15." (p. 170, 183)
+• [⑱] "young children should not be treated as 'mini-adults' as they have different needs and capacities, compared to older age players, in general." (p. 181)
+• [⑲] "The use of smaller playing areas seems to favour the increase of passing actions in older players while, in turn, increases in playing area appear to alter the available time for younger players to practice skills without the major constraint of pressing." (p. 183)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Nunes published version: 16 green highlights + matrix pages updated (170-184)
</commit_message>
<xml_diff>
--- a/LR_Matrix_v2.xlsx
+++ b/LR_Matrix_v2.xlsx
@@ -641,8 +641,8 @@
       <c r="G5" s="4" t="n"/>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>• [⑰] ★ "Results showed higher values in the large playing area for under-11 in the distance covered in different speed zones, sprint number and RPE (all p &lt; .001) … Opposite, under-23s were able to perform more passing on smaller playing areas … The impact of different playing areas was reduced for the under-15." (p. 170, 183)
-• [⑱] "young children should not be treated as 'mini-adults' as they have different needs and capacities, compared to older age players, in general." (p. 181)
+          <t>• [⑰] ★ "Results showed higher values in the large playing area for under-11 in the distance covered in different speed zones, sprint number and RPE (all p &lt; .001) … Opposite, under-23s were able to perform more passing on smaller playing areas … The impact of different playing areas was reduced for the under-15." (p. 170, 180)
+• [⑱] "young children should not be treated as 'mini-adults' as they have different needs and capacities, compared to older age players." (p. 181)
 • [⑲] "The use of smaller playing areas seems to favour the increase of passing actions in older players while, in turn, increases in playing area appear to alter the available time for younger players to practice skills without the major constraint of pressing." (p. 183)</t>
         </is>
       </c>

</xml_diff>